<commit_message>
Update card & XL
</commit_message>
<xml_diff>
--- a/data/perangkat.xlsx
+++ b/data/perangkat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\GH\perangkat\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB29C65-8FC3-4663-8501-568195B1DCCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A4BA79-6A10-4D71-8324-1F1346FFFE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Temenggungan" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2726" uniqueCount="840">
   <si>
     <t>NO</t>
   </si>
@@ -1666,9 +1666,6 @@
     <t>1975-05-27</t>
   </si>
   <si>
-    <t>KEPALA DUSUN KEMBANG I</t>
-  </si>
-  <si>
     <t>PURWADI</t>
   </si>
   <si>
@@ -1744,9 +1741,6 @@
     <t>1980-09-04</t>
   </si>
   <si>
-    <t>KEPALA DUSUN BESARAN</t>
-  </si>
-  <si>
     <t>2010-11-15</t>
   </si>
   <si>
@@ -1756,9 +1750,6 @@
     <t>1982-07-23</t>
   </si>
   <si>
-    <t>KEPALA DUSUN TPA</t>
-  </si>
-  <si>
     <t>2011-12-20</t>
   </si>
   <si>
@@ -2225,9 +2216,6 @@
   </si>
   <si>
     <t>1985-07-26</t>
-  </si>
-  <si>
-    <t>KAUR KESRA</t>
   </si>
   <si>
     <t>141/01/816.07/2009</t>
@@ -2598,10 +2586,12 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2649,7 +2639,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2660,7 +2650,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4905,7 +4894,7 @@
         <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>539</v>
+        <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>427</v>
@@ -4937,19 +4926,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>541</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>542</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -4978,10 +4967,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>542</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>543</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>544</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -5019,10 +5008,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>545</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>546</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -5031,7 +5020,7 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -5060,19 +5049,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>548</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>549</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>550</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -5101,19 +5090,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>552</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>553</v>
-      </c>
       <c r="F8" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -5142,19 +5131,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>555</v>
-      </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>161</v>
+        <v>72</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -5183,19 +5172,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>555</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>558</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>559</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -5224,16 +5213,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>561</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>562</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>278</v>
@@ -5265,19 +5254,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>563</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>564</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>565</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>566</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -5306,19 +5295,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>565</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>567</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>570</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -5347,19 +5336,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>573</v>
+        <v>57</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -5470,582 +5459,582 @@
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A2" s="6">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G2" s="6" t="s">
+      <c r="D3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>820</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>821</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>823</v>
+      </c>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="H6" s="4"/>
+      <c r="I6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>594</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>599</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>812</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>824</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>825</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A3" s="6">
-        <v>2</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>576</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>577</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>824</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>825</v>
-      </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A4" s="6">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="F11" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>580</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="H11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4"/>
+      <c r="Q11" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>826</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>827</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A5" s="6">
-        <v>4</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>583</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>584</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>585</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M5" s="6"/>
-      <c r="N5" s="6"/>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A6" s="6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>587</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>588</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>589</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>590</v>
-      </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>591</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A7" s="6">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>593</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>594</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>591</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A8" s="6">
-        <v>7</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>597</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>598</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>599</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>282</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>590</v>
-      </c>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>591</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A9" s="6">
-        <v>8</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>600</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A10" s="6">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>816</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>582</v>
-      </c>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>591</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A11" s="6">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="D12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>822</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>828</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="H12" s="4"/>
+      <c r="I12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>829</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>578</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>582</v>
-      </c>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A12" s="6">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="D13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>830</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="G13" s="4" t="s">
         <v>831</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>826</v>
-      </c>
-      <c r="G12" s="6" t="s">
+      <c r="H13" s="4"/>
+      <c r="I13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K13" s="4"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>832</v>
       </c>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J12" s="6" t="s">
+      <c r="C14" s="4" t="s">
+        <v>833</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>834</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>835</v>
+      </c>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A13" s="6">
-        <v>12</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>833</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>834</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>835</v>
-      </c>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A14" s="6">
-        <v>13</v>
-      </c>
-      <c r="B14" s="6" t="s">
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4"/>
+      <c r="Q14" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>836</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>837</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" s="6" t="s">
+      <c r="D15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F15" s="4" t="s">
         <v>838</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G15" s="4" t="s">
         <v>839</v>
       </c>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" s="6" t="s">
+      <c r="H15" s="4"/>
+      <c r="I15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J15" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A15" s="6">
-        <v>14</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>840</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>841</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>842</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>843</v>
-      </c>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6" t="s">
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4"/>
+      <c r="Q15" s="4" t="s">
         <v>25</v>
       </c>
     </row>
@@ -6140,10 +6129,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -6153,7 +6142,7 @@
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -6181,10 +6170,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -6194,7 +6183,7 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -6222,10 +6211,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -6235,7 +6224,7 @@
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -6263,10 +6252,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -6276,7 +6265,7 @@
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -6304,10 +6293,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -6317,7 +6306,7 @@
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -6345,10 +6334,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
@@ -6358,7 +6347,7 @@
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -6386,10 +6375,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -6399,7 +6388,7 @@
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -6427,10 +6416,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -6440,7 +6429,7 @@
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -6468,10 +6457,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>19</v>
@@ -6481,7 +6470,7 @@
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -6509,10 +6498,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>19</v>
@@ -6522,7 +6511,7 @@
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -6550,10 +6539,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
@@ -6563,7 +6552,7 @@
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -6591,20 +6580,20 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -6632,10 +6621,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -6645,7 +6634,7 @@
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -6759,10 +6748,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -6774,14 +6763,14 @@
         <v>411</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>87</v>
@@ -6800,10 +6789,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -6812,10 +6801,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -6841,10 +6830,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -6853,10 +6842,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -6882,10 +6871,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -6894,10 +6883,10 @@
         <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -6923,10 +6912,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -6935,10 +6924,10 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -6964,10 +6953,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
@@ -6976,17 +6965,17 @@
         <v>49</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>87</v>
@@ -7005,10 +6994,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -7017,10 +7006,10 @@
         <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -7046,10 +7035,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -7058,10 +7047,10 @@
         <v>57</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -7087,22 +7076,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>673</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>674</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>675</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>677</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -7128,22 +7117,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>678</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>679</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>682</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -7169,22 +7158,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>683</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>684</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>685</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>686</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -7210,22 +7199,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>686</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>687</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>688</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>689</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>690</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -7251,10 +7240,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -7263,10 +7252,10 @@
         <v>158</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -7292,10 +7281,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>19</v>
@@ -7304,10 +7293,10 @@
         <v>161</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -7333,22 +7322,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>278</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
@@ -7374,29 +7363,29 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>87</v>
@@ -7415,10 +7404,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>19</v>
@@ -7430,7 +7419,7 @@
         <v>427</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
@@ -7542,22 +7531,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>707</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>708</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>709</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>710</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -7585,10 +7574,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -7597,10 +7586,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -7628,10 +7617,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -7640,10 +7629,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -7671,22 +7660,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>720</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>721</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>722</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>723</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -7714,22 +7703,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>726</v>
+        <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>727</v>
+        <v>723</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -7757,10 +7746,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>728</v>
+        <v>724</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>56</v>
@@ -7769,10 +7758,10 @@
         <v>57</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -7800,10 +7789,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>730</v>
+        <v>726</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>731</v>
+        <v>727</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -7812,10 +7801,10 @@
         <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -7843,10 +7832,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>735</v>
+        <v>731</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -7855,10 +7844,10 @@
         <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>733</v>
+        <v>729</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -7886,22 +7875,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>736</v>
+        <v>732</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>737</v>
+        <v>733</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>738</v>
+        <v>734</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -7929,22 +7918,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>739</v>
+        <v>735</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>740</v>
+        <v>736</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>741</v>
+        <v>737</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>742</v>
+        <v>738</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -7972,22 +7961,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>741</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>742</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>743</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>745</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>746</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>747</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -8015,22 +8004,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>746</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>747</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>748</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>749</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>750</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>751</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>752</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -8058,10 +8047,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>753</v>
+        <v>749</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>754</v>
+        <v>750</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -8070,10 +8059,10 @@
         <v>72</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>755</v>
+        <v>751</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -8101,10 +8090,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>756</v>
+        <v>752</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>757</v>
+        <v>753</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>19</v>
@@ -8114,7 +8103,7 @@
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>758</v>
+        <v>754</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -8228,10 +8217,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>759</v>
+        <v>755</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>760</v>
+        <v>756</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -8273,10 +8262,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>761</v>
+        <v>757</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -8286,10 +8275,10 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>23</v>
@@ -8319,7 +8308,7 @@
         <v>191</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -8328,13 +8317,13 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>20</v>
@@ -8361,10 +8350,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -8373,13 +8362,13 @@
         <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>20</v>
@@ -8406,10 +8395,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -8418,13 +8407,13 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
@@ -8451,10 +8440,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>56</v>
@@ -8463,13 +8452,13 @@
         <v>57</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
@@ -8496,10 +8485,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -8508,13 +8497,13 @@
         <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>20</v>
@@ -8541,7 +8530,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
       <c r="C9" s="3">
         <v>27801</v>
@@ -8553,13 +8542,13 @@
         <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>20</v>
@@ -8586,25 +8575,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>778</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>779</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>780</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>781</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>782</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>783</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>784</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>785</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>786</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>20</v>
@@ -8631,25 +8620,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -8676,25 +8665,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -8721,10 +8710,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>793</v>
+        <v>789</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>794</v>
+        <v>790</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>19</v>
@@ -8733,13 +8722,13 @@
         <v>72</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>20</v>
@@ -8766,25 +8755,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>796</v>
+        <v>792</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>20</v>
@@ -8811,25 +8800,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>20</v>
@@ -8856,25 +8845,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>20</v>
@@ -8901,25 +8890,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>802</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>804</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>805</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>806</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>807</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>808</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>20</v>
@@ -8946,25 +8935,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>809</v>
+        <v>805</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>810</v>
+        <v>806</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>811</v>
+        <v>807</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>812</v>
+        <v>808</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>20</v>
@@ -8991,25 +8980,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>20</v>
@@ -11332,7 +11321,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>250</v>
@@ -12096,7 +12085,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>821</v>
+        <v>817</v>
       </c>
       <c r="C6" s="3">
         <v>36774</v>
@@ -12108,13 +12097,13 @@
         <v>52</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
@@ -12313,13 +12302,13 @@
         <v>161</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -12337,7 +12326,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>818</v>
+        <v>814</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>316</v>
@@ -12349,13 +12338,13 @@
         <v>317</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>819</v>
+        <v>815</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>820</v>
+        <v>816</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -12419,22 +12408,26 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>822</v>
+        <v>818</v>
       </c>
       <c r="C14" s="3">
-        <v>24222</v>
+        <v>32258</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>823</v>
+        <v>819</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
@@ -13265,7 +13258,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>817</v>
+        <v>813</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>373</v>

</xml_diff>

<commit_message>
Update foto & XL
</commit_message>
<xml_diff>
--- a/data/perangkat.xlsx
+++ b/data/perangkat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\GH\perangkat\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6A4BA79-6A10-4D71-8324-1F1346FFFE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{038FD497-BA1B-4DAB-A8C0-D251EC4D6F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Temenggungan" sheetId="1" r:id="rId1"/>
@@ -1522,9 +1522,6 @@
     <t>141/03/426.415.10/2026</t>
   </si>
   <si>
-    <t>ACHMAD MUFID MRTADHO</t>
-  </si>
-  <si>
     <t>MUSTAFA</t>
   </si>
   <si>
@@ -2567,6 +2564,9 @@
   </si>
   <si>
     <t>141/03/426.415.13/2024</t>
+  </si>
+  <si>
+    <t>ACHMAD MUFID MURTADHO</t>
   </si>
 </sst>
 </file>
@@ -2639,7 +2639,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2650,6 +2650,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4156,7 +4157,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>491</v>
+        <v>839</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>488</v>
@@ -4283,22 +4284,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>493</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>494</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>495</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -4326,10 +4327,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>496</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>497</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -4338,10 +4339,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>498</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>499</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -4369,10 +4370,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>500</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>501</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -4381,10 +4382,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -4412,10 +4413,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>504</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>505</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -4424,10 +4425,10 @@
         <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>506</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>507</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -4455,10 +4456,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>508</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>509</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -4467,10 +4468,10 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -4498,10 +4499,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>511</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>512</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
@@ -4510,10 +4511,10 @@
         <v>57</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>513</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>514</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -4541,10 +4542,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>515</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>516</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -4553,10 +4554,10 @@
         <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>517</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>518</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -4584,10 +4585,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>519</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>520</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -4596,10 +4597,10 @@
         <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -4627,10 +4628,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>522</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>523</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>19</v>
@@ -4639,10 +4640,10 @@
         <v>72</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>524</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -4670,22 +4671,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>529</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -4713,22 +4714,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>533</v>
-      </c>
       <c r="G12" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -4842,10 +4843,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>535</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -4857,7 +4858,7 @@
         <v>173</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -4885,10 +4886,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>538</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -4926,10 +4927,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>539</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>540</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -4938,7 +4939,7 @@
         <v>49</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -4967,10 +4968,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>542</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>543</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -5008,10 +5009,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>544</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>545</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -5020,7 +5021,7 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -5049,19 +5050,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -5090,19 +5091,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>552</v>
-      </c>
       <c r="F8" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -5131,10 +5132,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>553</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>554</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -5143,7 +5144,7 @@
         <v>72</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -5172,19 +5173,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>557</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>558</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -5213,16 +5214,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>559</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>560</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>561</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>278</v>
@@ -5254,10 +5255,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>562</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
@@ -5266,7 +5267,7 @@
         <v>52</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -5295,10 +5296,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>565</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>566</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>19</v>
@@ -5307,7 +5308,7 @@
         <v>34</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -5336,10 +5337,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>568</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>569</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -5348,7 +5349,7 @@
         <v>57</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -5463,9 +5464,11 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="C2" s="4"/>
+        <v>570</v>
+      </c>
+      <c r="C2" s="6">
+        <v>29183</v>
+      </c>
       <c r="D2" s="4" t="s">
         <v>19</v>
       </c>
@@ -5476,7 +5479,7 @@
         <v>173</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4" t="s">
@@ -5504,10 +5507,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>573</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>574</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>19</v>
@@ -5516,10 +5519,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>819</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>820</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>821</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4" t="s">
@@ -5547,10 +5550,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>576</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>577</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>19</v>
@@ -5559,10 +5562,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>821</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>822</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>823</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
@@ -5590,10 +5593,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>580</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>581</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>19</v>
@@ -5602,10 +5605,10 @@
         <v>72</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>582</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>583</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4" t="s">
@@ -5633,29 +5636,29 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>584</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>585</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>586</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>282</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4" t="s">
         <v>20</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>87</v>
@@ -5676,29 +5679,29 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>589</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>590</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>591</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>592</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>593</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4" t="s">
         <v>20</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>87</v>
@@ -5719,29 +5722,29 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>595</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>596</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>282</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4" t="s">
         <v>20</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>87</v>
@@ -5762,22 +5765,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>599</v>
-      </c>
       <c r="F9" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>592</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>593</v>
       </c>
       <c r="H9" s="4"/>
       <c r="I9" s="4" t="s">
@@ -5805,29 +5808,29 @@
         <v>9</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>599</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>601</v>
-      </c>
       <c r="D10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="F10" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>578</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>579</v>
       </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4" t="s">
         <v>20</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>87</v>
@@ -5848,22 +5851,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>823</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>824</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>825</v>
-      </c>
       <c r="D11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="F11" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>578</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>579</v>
       </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4" t="s">
@@ -5887,10 +5890,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>825</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>826</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>827</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>19</v>
@@ -5899,10 +5902,10 @@
         <v>49</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="H12" s="4"/>
       <c r="I12" s="4" t="s">
@@ -5929,7 +5932,7 @@
         <v>193</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>19</v>
@@ -5938,10 +5941,10 @@
         <v>52</v>
       </c>
       <c r="F13" s="4" t="s">
+        <v>829</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>830</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>831</v>
       </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4" t="s">
@@ -5965,10 +5968,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>831</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>832</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>833</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>56</v>
@@ -5977,10 +5980,10 @@
         <v>80</v>
       </c>
       <c r="F14" s="4" t="s">
+        <v>833</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>834</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>835</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="4" t="s">
@@ -6004,10 +6007,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>835</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>836</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>837</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>19</v>
@@ -6016,10 +6019,10 @@
         <v>80</v>
       </c>
       <c r="F15" s="4" t="s">
+        <v>837</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>838</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>839</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
@@ -6129,10 +6132,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>602</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>603</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -6142,7 +6145,7 @@
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -6170,10 +6173,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>605</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>606</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -6183,7 +6186,7 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -6211,10 +6214,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>608</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>609</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -6224,7 +6227,7 @@
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -6252,10 +6255,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>612</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -6265,7 +6268,7 @@
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -6293,10 +6296,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>614</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>615</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -6306,7 +6309,7 @@
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -6334,10 +6337,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>616</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>617</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
@@ -6347,7 +6350,7 @@
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -6375,10 +6378,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>619</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>620</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -6388,7 +6391,7 @@
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -6416,10 +6419,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>622</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>623</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -6429,7 +6432,7 @@
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -6457,10 +6460,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>19</v>
@@ -6470,7 +6473,7 @@
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -6498,10 +6501,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>627</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>628</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>19</v>
@@ -6511,7 +6514,7 @@
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -6539,10 +6542,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>630</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>631</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>19</v>
@@ -6552,7 +6555,7 @@
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -6580,20 +6583,20 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>633</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>634</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>635</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -6621,10 +6624,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>637</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>638</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -6634,7 +6637,7 @@
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -6748,10 +6751,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>640</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>641</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -6763,14 +6766,14 @@
         <v>411</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>87</v>
@@ -6789,10 +6792,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>644</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>645</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -6801,10 +6804,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>646</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>647</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -6830,10 +6833,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>648</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>649</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -6842,10 +6845,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>650</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>651</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -6871,10 +6874,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -6883,10 +6886,10 @@
         <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>653</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>654</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -6912,10 +6915,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>655</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>656</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -6924,10 +6927,10 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>657</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>658</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -6953,10 +6956,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>659</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>660</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>19</v>
@@ -6965,17 +6968,17 @@
         <v>49</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>661</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>662</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>87</v>
@@ -6994,10 +6997,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>664</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>665</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -7006,10 +7009,10 @@
         <v>52</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -7035,10 +7038,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>667</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>668</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -7047,10 +7050,10 @@
         <v>57</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -7076,22 +7079,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>670</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>671</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>672</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>673</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>674</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -7117,22 +7120,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>675</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>676</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>677</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -7158,22 +7161,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>680</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>681</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>682</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>567</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>683</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -7199,22 +7202,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>683</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>686</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>661</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>687</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -7240,10 +7243,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>687</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>688</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>689</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -7252,10 +7255,10 @@
         <v>158</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -7281,10 +7284,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>690</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>691</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>19</v>
@@ -7293,10 +7296,10 @@
         <v>161</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -7322,22 +7325,22 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>693</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>694</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>695</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>278</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
@@ -7363,29 +7366,29 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>697</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>698</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>699</v>
-      </c>
       <c r="F17" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>679</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>87</v>
@@ -7404,10 +7407,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>700</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>701</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>702</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>19</v>
@@ -7419,7 +7422,7 @@
         <v>427</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
@@ -7531,22 +7534,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>704</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>705</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>706</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>707</v>
       </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
@@ -7574,10 +7577,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>708</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>709</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -7586,10 +7589,10 @@
         <v>28</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>710</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>711</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
@@ -7617,10 +7620,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>712</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>713</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -7629,10 +7632,10 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>714</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>715</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
@@ -7660,22 +7663,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>716</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>717</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>719</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>720</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
@@ -7703,10 +7706,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>720</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>721</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>722</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -7715,10 +7718,10 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
@@ -7746,10 +7749,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>724</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>725</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>56</v>
@@ -7758,10 +7761,10 @@
         <v>57</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>719</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>720</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
@@ -7789,10 +7792,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>725</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>726</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>727</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -7801,10 +7804,10 @@
         <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>728</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>729</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
@@ -7832,10 +7835,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>729</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>730</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>731</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>19</v>
@@ -7844,10 +7847,10 @@
         <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>728</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>729</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
@@ -7875,22 +7878,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>732</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>733</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>734</v>
-      </c>
       <c r="F10" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>719</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>720</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
@@ -7918,22 +7921,22 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>735</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>736</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>737</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>738</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
@@ -7961,22 +7964,22 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>738</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>739</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>740</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>741</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>742</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>743</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
@@ -8004,22 +8007,22 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>743</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>744</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>745</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>746</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>747</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>748</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
@@ -8047,10 +8050,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>749</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>750</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>19</v>
@@ -8059,10 +8062,10 @@
         <v>72</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -8090,10 +8093,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>752</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>753</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>19</v>
@@ -8103,7 +8106,7 @@
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
@@ -8217,10 +8220,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>755</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>756</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
@@ -8262,10 +8265,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>756</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>757</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>758</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>19</v>
@@ -8275,10 +8278,10 @@
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>759</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>760</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>23</v>
@@ -8308,7 +8311,7 @@
         <v>191</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>19</v>
@@ -8317,13 +8320,13 @@
         <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>762</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>763</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>764</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>20</v>
@@ -8350,10 +8353,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>765</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>766</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>19</v>
@@ -8362,13 +8365,13 @@
         <v>44</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G5" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>759</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>760</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>20</v>
@@ -8395,10 +8398,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>767</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>768</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
@@ -8407,13 +8410,13 @@
         <v>39</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
@@ -8440,10 +8443,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>769</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>770</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>771</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>56</v>
@@ -8452,13 +8455,13 @@
         <v>57</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>20</v>
@@ -8485,10 +8488,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>773</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>774</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>19</v>
@@ -8497,13 +8500,13 @@
         <v>49</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G8" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>775</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>776</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>20</v>
@@ -8530,7 +8533,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C9" s="3">
         <v>27801</v>
@@ -8542,13 +8545,13 @@
         <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>20</v>
@@ -8575,25 +8578,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>777</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>778</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>779</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>780</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>762</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>781</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>782</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>20</v>
@@ -8620,25 +8623,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>782</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>783</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>784</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>741</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>762</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>785</v>
-      </c>
       <c r="H11" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -8665,25 +8668,25 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>785</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>786</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>787</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>788</v>
-      </c>
       <c r="F12" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -8710,10 +8713,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>788</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>789</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>790</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>19</v>
@@ -8722,13 +8725,13 @@
         <v>72</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G13" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>759</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>760</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>20</v>
@@ -8755,25 +8758,25 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>791</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>792</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>793</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>20</v>
@@ -8800,25 +8803,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>793</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>794</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>795</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>796</v>
-      </c>
       <c r="F15" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>759</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>760</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>20</v>
@@ -8845,25 +8848,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>796</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>797</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>798</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>799</v>
-      </c>
       <c r="F16" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>20</v>
@@ -8890,25 +8893,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>800</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>801</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>802</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>762</v>
-      </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>803</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>804</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>20</v>
@@ -8935,25 +8938,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>805</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>806</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>761</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>807</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>762</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>808</v>
-      </c>
       <c r="H18" s="2" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>20</v>
@@ -8980,25 +8983,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>809</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>810</v>
-      </c>
       <c r="D19" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>20</v>
@@ -11321,7 +11324,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>250</v>
@@ -12085,7 +12088,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C6" s="3">
         <v>36774</v>
@@ -12097,13 +12100,13 @@
         <v>52</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>815</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>816</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>20</v>
@@ -12302,13 +12305,13 @@
         <v>161</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>815</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>816</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>20</v>
@@ -12326,7 +12329,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>316</v>
@@ -12338,13 +12341,13 @@
         <v>317</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="G12" s="2" t="s">
+        <v>814</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>815</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>816</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>20</v>
@@ -12408,7 +12411,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="C14" s="3">
         <v>32258</v>
@@ -12417,7 +12420,7 @@
         <v>19</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -13258,7 +13261,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>373</v>

</xml_diff>